<commit_message>
Implemented AI-routing (Claude) hybrid automation with Playwright
</commit_message>
<xml_diff>
--- a/Excel Sheets/Cert Test.xlsx
+++ b/Excel Sheets/Cert Test.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,12 +466,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>New York State University</t>
+          <t>State University of New York</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>New York City, New York</t>
+          <t>Albany, New York</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -479,22 +479,24 @@
           <t>Board Medical Certification</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>321987</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>321987</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>12-31-2024</t>
+          <t>State University of New York Albany</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Verified via DAPIP</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>06-07-2026</t>
+          <t>06-08-2026 @ 08:51PM</t>
         </is>
       </c>
     </row>
@@ -511,7 +513,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Sacramento, California</t>
+          <t>Los Angeles, California</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -519,142 +521,108 @@
           <t>Certification of Completion in Medicine</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v>524689</v>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>524689</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>12-31-2024</t>
+          <t>California State University Los Angeles</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Verified via DAPIP</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>06-07-2026</t>
+          <t>06-08-2026 @ 08:51PM</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Punch Rocks</t>
+          <t>Taki Omaoi</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Money Banks University </t>
+          <t>Japan Culinary Institute</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Augusta, Maine</t>
+          <t>Tokyo, Japan</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Computer Engineer Certification in Robotics</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>578799</v>
+          <t>Certification of Food Safety in Japan</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>879342</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>12-31-2024</t>
+          <t>Japan Culinary Institute Tokyo</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Verified via International Registry</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>06-07-2026</t>
+          <t>06-08-2026 @ 08:51PM</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Taki Omaoi</t>
+          <t>Jess Toicana</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Japan Institute of Culinary Arts</t>
+          <t>Culinary Institute of America</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Tokyo, Japan</t>
+          <t>Hyde Park, New York</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Certification of Food Safety in Japan</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>879342</v>
+          <t>Certification of Raw Food Handling</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>369875</t>
+        </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>12-31-2024</t>
+          <t>Culinary Institute of America</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Verified via DAPIP</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>06-07-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Jess Toicana</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Culinary Arts Institute of New York</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>New York City, New York</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Certification of Raw Food Handling</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>369875</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>12-31-2024</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>06-07-2026</t>
+          <t>06-08-2026 @ 08:51PM</t>
         </is>
       </c>
     </row>

</xml_diff>